<commit_message>
Updating results for iteration 7
</commit_message>
<xml_diff>
--- a/results/results_iter7.xlsx
+++ b/results/results_iter7.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danemerson/Documents/CMU/01_Research/Projects/CPA/Bayesian Optimization/cpa-bayesian-opt/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8387EEC8-ADD8-174F-BA7E-D9118B9EE121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2517B2E0-8B7F-8941-88B5-1B795724B945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="26000" windowHeight="26360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="19980" xr2:uid="{5BBBF348-0167-5541-B79A-EC4E010FEC1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -65,6 +68,9 @@
     <t>Predicted Viability</t>
   </si>
   <si>
+    <t>n2</t>
+  </si>
+  <si>
     <t>Random 1</t>
   </si>
   <si>
@@ -185,19 +191,16 @@
     <t>VarLogNEHVI 10</t>
   </si>
   <si>
-    <t>n1</t>
-  </si>
-  <si>
-    <t>n2</t>
+    <t>n3</t>
+  </si>
+  <si>
+    <t>n4 (6.16.25)</t>
   </si>
   <si>
     <t>Experimental average</t>
   </si>
   <si>
     <t>SD</t>
-  </si>
-  <si>
-    <t>n3</t>
   </si>
 </sst>
 </file>
@@ -206,7 +209,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -233,7 +236,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -256,22 +259,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -284,9 +307,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -294,44 +317,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -358,14 +381,32 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -392,9 +433,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -403,230 +462,204 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E45FE471-5B82-B44F-A985-1EBE7A3CBEB8}">
   <dimension ref="A1:P41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19" customWidth="1"/>
+    <col min="10" max="11" width="17.5" customWidth="1"/>
+    <col min="15" max="15" width="19.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
-        <v>50</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="L1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" t="s">
         <v>54</v>
       </c>
-      <c r="O1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P1" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>10</v>
+      <c r="A2" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="B2">
         <v>0.5</v>
@@ -652,30 +685,30 @@
       <c r="I2">
         <v>5.5</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>29.946421811653249</v>
       </c>
-      <c r="L2">
-        <v>34.210590088452697</v>
-      </c>
-      <c r="M2">
+      <c r="L2" s="4">
         <v>41.802114565251685</v>
       </c>
-      <c r="N2">
+      <c r="M2" s="4">
         <v>37.043386522484504</v>
       </c>
-      <c r="O2" s="2">
-        <f t="shared" ref="O2:O41" si="0">AVERAGE(L2:N2)</f>
-        <v>37.685363725396293</v>
-      </c>
-      <c r="P2">
-        <f t="shared" ref="P2:P41" si="1">_xlfn.STDEV.P(L2:N2)</f>
-        <v>3.1322954327727315</v>
+      <c r="N2" s="4">
+        <v>38.518767824562033</v>
+      </c>
+      <c r="O2" s="1">
+        <f>AVERAGE(L2:N2)</f>
+        <v>39.121422970766069</v>
+      </c>
+      <c r="P2" s="4">
+        <f>_xlfn.STDEV.P(L2:N2)</f>
+        <v>1.98893071191354</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>11</v>
+      <c r="A3" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="B3">
         <v>0.5</v>
@@ -701,30 +734,30 @@
       <c r="I3">
         <v>5</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>28.30354088266154</v>
       </c>
-      <c r="L3">
-        <v>35.344723130982686</v>
-      </c>
-      <c r="M3">
+      <c r="L3" s="4">
         <v>45.778759665456825</v>
       </c>
-      <c r="N3">
+      <c r="M3" s="4">
         <v>50.652775946195433</v>
       </c>
-      <c r="O3" s="2">
-        <f t="shared" si="0"/>
-        <v>43.925419580878305</v>
-      </c>
-      <c r="P3">
-        <f t="shared" si="1"/>
-        <v>6.3854142308945603</v>
+      <c r="N3" s="4">
+        <v>51.017660708908302</v>
+      </c>
+      <c r="O3" s="1">
+        <f t="shared" ref="O3:O41" si="0">AVERAGE(L3:N3)</f>
+        <v>49.14973210685352</v>
+      </c>
+      <c r="P3" s="4">
+        <f t="shared" ref="P3:P40" si="1">_xlfn.STDEV.P(L3:N3)</f>
+        <v>2.3882876184981021</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>12</v>
+      <c r="A4" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -750,30 +783,30 @@
       <c r="I4">
         <v>6</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>34.329584073668521</v>
       </c>
-      <c r="L4">
-        <v>47.035017569368719</v>
-      </c>
-      <c r="M4">
+      <c r="L4" s="4">
         <v>34.254604477107229</v>
       </c>
-      <c r="N4">
+      <c r="M4" s="4">
         <v>25.96597652644072</v>
       </c>
-      <c r="O4" s="2">
-        <f t="shared" si="0"/>
-        <v>35.75186619097223</v>
-      </c>
-      <c r="P4">
-        <f t="shared" si="1"/>
-        <v>8.6663128298409973</v>
+      <c r="N4" s="4">
+        <v>16.008006660407773</v>
+      </c>
+      <c r="O4" s="1">
+        <f t="shared" si="0"/>
+        <v>25.409529221318575</v>
+      </c>
+      <c r="P4" s="4">
+        <f t="shared" si="1"/>
+        <v>7.4595267130307308</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>13</v>
+      <c r="A5" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="B5">
         <v>2.5</v>
@@ -799,30 +832,30 @@
       <c r="I5">
         <v>6</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>57.676995630625953</v>
       </c>
-      <c r="L5">
-        <v>51.658790742760218</v>
-      </c>
-      <c r="M5">
+      <c r="L5" s="4">
         <v>66.311233346107883</v>
       </c>
-      <c r="N5">
+      <c r="M5" s="4">
         <v>67.585388368719507</v>
       </c>
-      <c r="O5" s="2">
-        <f t="shared" si="0"/>
-        <v>61.851804152529205</v>
-      </c>
-      <c r="P5">
-        <f t="shared" si="1"/>
-        <v>7.2262950181592709</v>
+      <c r="N5" s="4">
+        <v>67.342745292544251</v>
+      </c>
+      <c r="O5" s="1">
+        <f t="shared" si="0"/>
+        <v>67.079789002457218</v>
+      </c>
+      <c r="P5" s="4">
+        <f t="shared" si="1"/>
+        <v>0.55240520350183775</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
+      <c r="A6" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -848,30 +881,30 @@
       <c r="I6">
         <v>5.5</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45.447783731164108</v>
       </c>
-      <c r="L6">
-        <v>63.349085181146265</v>
-      </c>
-      <c r="M6">
+      <c r="L6" s="4">
         <v>63.714240627606557</v>
       </c>
-      <c r="N6">
+      <c r="M6" s="4">
         <v>58.327838586311486</v>
       </c>
-      <c r="O6" s="2">
-        <f t="shared" si="0"/>
-        <v>61.797054798354772</v>
-      </c>
-      <c r="P6">
-        <f t="shared" si="1"/>
-        <v>2.4576317149439979</v>
+      <c r="N6" s="4">
+        <v>59.690361893964891</v>
+      </c>
+      <c r="O6" s="1">
+        <f t="shared" si="0"/>
+        <v>60.577480369294314</v>
+      </c>
+      <c r="P6" s="4">
+        <f t="shared" si="1"/>
+        <v>2.2867103197344467</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>15</v>
+      <c r="A7" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -897,30 +930,30 @@
       <c r="I7">
         <v>5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>47.993203590528267</v>
       </c>
-      <c r="L7">
-        <v>52.618441778747133</v>
-      </c>
-      <c r="M7">
+      <c r="L7" s="4">
         <v>77.67307648955115</v>
       </c>
-      <c r="N7">
+      <c r="M7" s="4">
         <v>71.541606224449424</v>
       </c>
-      <c r="O7" s="2">
-        <f t="shared" si="0"/>
-        <v>67.277708164249233</v>
-      </c>
-      <c r="P7">
-        <f t="shared" si="1"/>
-        <v>10.663623528106816</v>
+      <c r="N7" s="4">
+        <v>74.548739659539791</v>
+      </c>
+      <c r="O7" s="1">
+        <f t="shared" si="0"/>
+        <v>74.587807457846779</v>
+      </c>
+      <c r="P7" s="4">
+        <f t="shared" si="1"/>
+        <v>2.5033146855859032</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>16</v>
+      <c r="A8" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="B8">
         <v>0.5</v>
@@ -946,30 +979,30 @@
       <c r="I8">
         <v>6</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>1.578545185350102</v>
       </c>
-      <c r="L8">
-        <v>-0.94753422997697834</v>
-      </c>
-      <c r="M8">
+      <c r="L8" s="4">
         <v>-0.72364120020739897</v>
       </c>
-      <c r="N8">
+      <c r="M8" s="4">
         <v>-0.61980746406435483</v>
       </c>
-      <c r="O8" s="2">
-        <f t="shared" si="0"/>
-        <v>-0.76366096474957734</v>
-      </c>
-      <c r="P8">
-        <f t="shared" si="1"/>
-        <v>0.13675377981222447</v>
+      <c r="N8" s="4">
+        <v>-0.25330806157334435</v>
+      </c>
+      <c r="O8" s="1">
+        <f t="shared" si="0"/>
+        <v>-0.53225224194836607</v>
+      </c>
+      <c r="P8" s="4">
+        <f t="shared" si="1"/>
+        <v>0.20174695869525161</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>17</v>
+      <c r="A9" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="B9">
         <v>0.5</v>
@@ -995,30 +1028,30 @@
       <c r="I9">
         <v>5.5</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>35.496055760121493</v>
       </c>
-      <c r="L9">
-        <v>41.364352356718783</v>
-      </c>
-      <c r="M9">
+      <c r="L9" s="4">
         <v>47.077256024707488</v>
       </c>
-      <c r="N9">
+      <c r="M9" s="4">
         <v>34.353158380588155</v>
       </c>
-      <c r="O9" s="2">
-        <f t="shared" si="0"/>
-        <v>40.93158892067148</v>
-      </c>
-      <c r="P9">
-        <f t="shared" si="1"/>
-        <v>5.2035967277743094</v>
+      <c r="N9" s="4">
+        <v>35.840433635059256</v>
+      </c>
+      <c r="O9" s="1">
+        <f t="shared" si="0"/>
+        <v>39.0902826801183</v>
+      </c>
+      <c r="P9" s="4">
+        <f t="shared" si="1"/>
+        <v>5.6801880441891726</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>18</v>
+      <c r="A10" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="B10">
         <v>0.5</v>
@@ -1044,30 +1077,30 @@
       <c r="I10">
         <v>6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>17.745978700594559</v>
       </c>
-      <c r="L10">
-        <v>11.527929237852904</v>
-      </c>
-      <c r="M10">
+      <c r="L10" s="4">
         <v>22.405825198944971</v>
       </c>
-      <c r="N10">
+      <c r="M10" s="4">
         <v>17.024924172491097</v>
       </c>
-      <c r="O10" s="2">
-        <f t="shared" si="0"/>
-        <v>16.986226203096326</v>
-      </c>
-      <c r="P10">
-        <f t="shared" si="1"/>
-        <v>4.4409667329469471</v>
+      <c r="N10" s="4">
+        <v>14.094910810762936</v>
+      </c>
+      <c r="O10" s="1">
+        <f t="shared" si="0"/>
+        <v>17.841886727399668</v>
+      </c>
+      <c r="P10" s="4">
+        <f t="shared" si="1"/>
+        <v>3.4417432941282224</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>19</v>
+      <c r="A11" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1093,30 +1126,30 @@
       <c r="I11">
         <v>5.5</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>11.4845069177057</v>
       </c>
-      <c r="L11">
-        <v>17.111353447231316</v>
-      </c>
-      <c r="M11">
+      <c r="L11" s="4">
         <v>24.840505872539953</v>
       </c>
-      <c r="N11">
+      <c r="M11" s="4">
         <v>19.240406171699853</v>
       </c>
-      <c r="O11" s="2">
-        <f t="shared" si="0"/>
-        <v>20.397421830490376</v>
-      </c>
-      <c r="P11">
-        <f t="shared" si="1"/>
-        <v>3.2597508319326454</v>
+      <c r="N11" s="4">
+        <v>21.428444901068151</v>
+      </c>
+      <c r="O11" s="1">
+        <f t="shared" si="0"/>
+        <v>21.836452315102651</v>
+      </c>
+      <c r="P11" s="4">
+        <f t="shared" si="1"/>
+        <v>2.3043627755871583</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>20</v>
+      <c r="A12" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="B12">
         <v>0.5</v>
@@ -1142,30 +1175,30 @@
       <c r="I12">
         <v>6</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>60.374211549335691</v>
       </c>
-      <c r="L12">
-        <v>71.288016478856193</v>
-      </c>
-      <c r="M12">
+      <c r="L12" s="4">
         <v>72.479091052548512</v>
       </c>
-      <c r="N12">
+      <c r="M12" s="4">
         <v>79.37491757879468</v>
       </c>
-      <c r="O12" s="2">
-        <f t="shared" si="0"/>
-        <v>74.380675036733123</v>
-      </c>
-      <c r="P12">
-        <f t="shared" si="1"/>
-        <v>3.5647822361473134</v>
+      <c r="N12" s="4">
+        <v>69.44715072715357</v>
+      </c>
+      <c r="O12" s="1">
+        <f t="shared" si="0"/>
+        <v>73.767053119498925</v>
+      </c>
+      <c r="P12" s="4">
+        <f t="shared" si="1"/>
+        <v>4.154056120593733</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>21</v>
+      <c r="A13" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="B13">
         <v>3.5</v>
@@ -1191,30 +1224,30 @@
       <c r="I13">
         <v>6</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>54.748380943563681</v>
       </c>
-      <c r="L13">
-        <v>15.366533381800561</v>
-      </c>
-      <c r="M13">
+      <c r="L13" s="4">
         <v>42.938298879596012</v>
       </c>
-      <c r="N13">
+      <c r="M13" s="4">
         <v>52.235263088487407</v>
       </c>
-      <c r="O13" s="2">
-        <f t="shared" si="0"/>
-        <v>36.84669844996133</v>
-      </c>
-      <c r="P13">
-        <f t="shared" si="1"/>
-        <v>15.655808387345727</v>
+      <c r="N13" s="4">
+        <v>42.344959523851699</v>
+      </c>
+      <c r="O13" s="1">
+        <f t="shared" si="0"/>
+        <v>45.839507163978375</v>
+      </c>
+      <c r="P13" s="4">
+        <f t="shared" si="1"/>
+        <v>4.5289648031449072</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>22</v>
+      <c r="A14" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="B14">
         <v>3.5</v>
@@ -1240,30 +1273,30 @@
       <c r="I14">
         <v>6</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>58.850065996074832</v>
       </c>
-      <c r="L14">
-        <v>5.7700230219314204</v>
-      </c>
-      <c r="M14">
+      <c r="L14" s="4">
         <v>46.265695800175827</v>
       </c>
-      <c r="N14">
+      <c r="M14" s="4">
         <v>44.955822233944353</v>
       </c>
-      <c r="O14" s="2">
-        <f t="shared" si="0"/>
-        <v>32.330513685350532</v>
-      </c>
-      <c r="P14">
-        <f t="shared" si="1"/>
-        <v>18.788714527628162</v>
+      <c r="N14" s="4">
+        <v>46.362460808105865</v>
+      </c>
+      <c r="O14" s="1">
+        <f t="shared" si="0"/>
+        <v>45.861326280742013</v>
+      </c>
+      <c r="P14" s="4">
+        <f t="shared" si="1"/>
+        <v>0.64150554726888731</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>23</v>
+      <c r="A15" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="B15">
         <v>2.5</v>
@@ -1289,30 +1322,30 @@
       <c r="I15">
         <v>6</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46.975942311486627</v>
       </c>
-      <c r="L15">
-        <v>44.679510481037198</v>
-      </c>
-      <c r="M15">
+      <c r="L15" s="4">
         <v>39.529745936563039</v>
       </c>
-      <c r="N15">
+      <c r="M15" s="4">
         <v>21.535012528023209</v>
       </c>
-      <c r="O15" s="2">
-        <f t="shared" si="0"/>
-        <v>35.248089648541146</v>
-      </c>
-      <c r="P15">
-        <f t="shared" si="1"/>
-        <v>9.9219078071654216</v>
+      <c r="N15" s="4">
+        <v>42.663808832125838</v>
+      </c>
+      <c r="O15" s="1">
+        <f t="shared" si="0"/>
+        <v>34.576189098904031</v>
+      </c>
+      <c r="P15" s="4">
+        <f t="shared" si="1"/>
+        <v>9.3098443353618574</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>24</v>
+      <c r="A16" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="B16">
         <v>1.5</v>
@@ -1338,30 +1371,30 @@
       <c r="I16">
         <v>6</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>49.510512761545883</v>
       </c>
-      <c r="L16">
-        <v>59.248758027383992</v>
-      </c>
-      <c r="M16">
+      <c r="L16" s="4">
         <v>42.28905069997068</v>
       </c>
-      <c r="N16">
+      <c r="M16" s="4">
         <v>44.006329948569167</v>
       </c>
-      <c r="O16" s="2">
-        <f t="shared" si="0"/>
-        <v>48.514712891974618</v>
-      </c>
-      <c r="P16">
-        <f t="shared" si="1"/>
-        <v>7.6224254989765194</v>
+      <c r="N16" s="4">
+        <v>53.887304483375559</v>
+      </c>
+      <c r="O16" s="1">
+        <f t="shared" si="0"/>
+        <v>46.727561710638469</v>
+      </c>
+      <c r="P16" s="4">
+        <f t="shared" si="1"/>
+        <v>5.1110142133264214</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>25</v>
+      <c r="A17" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="B17">
         <v>4</v>
@@ -1387,30 +1420,30 @@
       <c r="I17">
         <v>6</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>53.027573489438034</v>
       </c>
-      <c r="L17">
-        <v>0.36108081909608669</v>
-      </c>
-      <c r="M17">
+      <c r="L17" s="4">
         <v>38.880497756937714</v>
       </c>
-      <c r="N17">
+      <c r="M17" s="4">
         <v>54.925491230383756</v>
       </c>
-      <c r="O17" s="2">
-        <f t="shared" si="0"/>
-        <v>31.389023268805854</v>
-      </c>
-      <c r="P17">
-        <f t="shared" si="1"/>
-        <v>22.897021107378535</v>
+      <c r="N17" s="4">
+        <v>41.005792429100318</v>
+      </c>
+      <c r="O17" s="1">
+        <f t="shared" si="0"/>
+        <v>44.937260472140593</v>
+      </c>
+      <c r="P17" s="4">
+        <f t="shared" si="1"/>
+        <v>7.1158407617941437</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>26</v>
+      <c r="A18" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -1436,30 +1469,30 @@
       <c r="I18">
         <v>6</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46.168789861672167</v>
       </c>
-      <c r="L18">
-        <v>34.036108081909617</v>
-      </c>
-      <c r="M18">
+      <c r="L18" s="4">
         <v>18.753804188552486</v>
       </c>
-      <c r="N18">
+      <c r="M18" s="4">
         <v>14.967690887511537</v>
       </c>
-      <c r="O18" s="2">
-        <f t="shared" si="0"/>
-        <v>22.585867719324551</v>
-      </c>
-      <c r="P18">
-        <f t="shared" si="1"/>
-        <v>8.242761137418654</v>
+      <c r="N18" s="4">
+        <v>11.480346482914994</v>
+      </c>
+      <c r="O18" s="1">
+        <f t="shared" si="0"/>
+        <v>15.067280519659674</v>
+      </c>
+      <c r="P18" s="4">
+        <f t="shared" si="1"/>
+        <v>2.9702115884279858</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>27</v>
+      <c r="A19" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="B19">
         <v>2</v>
@@ -1485,30 +1518,30 @@
       <c r="I19">
         <v>6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>44.263602067624397</v>
       </c>
-      <c r="L19">
-        <v>19.815824548648983</v>
-      </c>
-      <c r="M19">
+      <c r="L19" s="4">
         <v>13.64097477400302</v>
       </c>
-      <c r="N19">
+      <c r="M19" s="4">
         <v>12.435711459844388</v>
       </c>
-      <c r="O19" s="2">
-        <f t="shared" si="0"/>
-        <v>15.297503594165462</v>
-      </c>
-      <c r="P19">
-        <f t="shared" si="1"/>
-        <v>3.2326029862334269</v>
+      <c r="N19" s="4">
+        <v>14.03114094910811</v>
+      </c>
+      <c r="O19" s="1">
+        <f t="shared" si="0"/>
+        <v>13.369275727651839</v>
+      </c>
+      <c r="P19" s="4">
+        <f t="shared" si="1"/>
+        <v>0.67907490634646039</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>28</v>
+      <c r="A20" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -1534,30 +1567,30 @@
       <c r="I20">
         <v>5</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>57.406390616846167</v>
       </c>
-      <c r="L20">
-        <v>56.020840906337085</v>
-      </c>
-      <c r="M20">
+      <c r="L20" s="4">
         <v>52.920489641335458</v>
       </c>
-      <c r="N20">
+      <c r="M20" s="4">
         <v>66.556771726229726</v>
       </c>
-      <c r="O20" s="2">
-        <f t="shared" si="0"/>
-        <v>58.499367424634094</v>
-      </c>
-      <c r="P20">
-        <f t="shared" si="1"/>
-        <v>5.8363440355030587</v>
+      <c r="N20" s="4">
+        <v>63.580323454909404</v>
+      </c>
+      <c r="O20" s="1">
+        <f t="shared" si="0"/>
+        <v>61.01919494082486</v>
+      </c>
+      <c r="P20" s="4">
+        <f t="shared" si="1"/>
+        <v>5.854148484846438</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
-        <v>29</v>
+      <c r="A21" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1583,30 +1616,30 @@
       <c r="I21">
         <v>6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>24.23038488042765</v>
       </c>
-      <c r="L21">
-        <v>8.9106991397067752</v>
-      </c>
-      <c r="M21">
+      <c r="L21" s="4">
         <v>10.313577853423205</v>
       </c>
-      <c r="N21">
+      <c r="M21" s="4">
         <v>8.7959910325728607</v>
       </c>
-      <c r="O21" s="2">
-        <f t="shared" si="0"/>
-        <v>9.3400893419009474</v>
-      </c>
-      <c r="P21">
-        <f t="shared" si="1"/>
-        <v>0.68995139877623601</v>
+      <c r="N21" s="4">
+        <v>9.1846314633411872</v>
+      </c>
+      <c r="O21" s="1">
+        <f t="shared" si="0"/>
+        <v>9.4314001164457508</v>
+      </c>
+      <c r="P21" s="4">
+        <f t="shared" si="1"/>
+        <v>0.64365545432368487</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>30</v>
+      <c r="A22" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1632,30 +1665,30 @@
       <c r="I22">
         <v>2.5</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>91.320908352434571</v>
       </c>
-      <c r="L22">
-        <v>92.313098267296766</v>
-      </c>
-      <c r="M22">
+      <c r="L22" s="4">
         <v>88.223359408462741</v>
       </c>
-      <c r="N22">
+      <c r="M22" s="4">
         <v>89.265462218119481</v>
       </c>
-      <c r="O22" s="2">
-        <f t="shared" si="0"/>
-        <v>89.933973297959653</v>
-      </c>
-      <c r="P22">
-        <f t="shared" si="1"/>
-        <v>1.7352562310825208</v>
+      <c r="N22" s="4">
+        <v>86.473703788992623</v>
+      </c>
+      <c r="O22" s="1">
+        <f t="shared" si="0"/>
+        <v>87.987508471858291</v>
+      </c>
+      <c r="P22" s="4">
+        <f t="shared" si="1"/>
+        <v>1.1518674778732481</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
-        <v>31</v>
+      <c r="A23" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -1681,30 +1714,30 @@
       <c r="I23">
         <v>4.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>86.446409190518395</v>
       </c>
-      <c r="L23">
-        <v>111.06991397067735</v>
-      </c>
-      <c r="M23">
+      <c r="L23" s="4">
         <v>88.872607588088087</v>
       </c>
-      <c r="N23">
+      <c r="M23" s="4">
         <v>95.199789001714365</v>
       </c>
-      <c r="O23" s="2">
-        <f t="shared" si="0"/>
-        <v>98.380770186826609</v>
-      </c>
-      <c r="P23">
-        <f t="shared" si="1"/>
-        <v>9.3369903657678694</v>
+      <c r="N23" s="4">
+        <v>91.894142029652997</v>
+      </c>
+      <c r="O23" s="1">
+        <f t="shared" si="0"/>
+        <v>91.98884620648515</v>
+      </c>
+      <c r="P23" s="4">
+        <f t="shared" si="1"/>
+        <v>2.5839288975081529</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
-        <v>32</v>
+      <c r="A24" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -1730,30 +1763,30 @@
       <c r="I24">
         <v>5</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>84.58698943165632</v>
       </c>
-      <c r="L24">
-        <v>102.95650066642435</v>
-      </c>
-      <c r="M24">
+      <c r="L24" s="4">
         <v>92.28116053112106</v>
       </c>
-      <c r="N24">
+      <c r="M24" s="4">
         <v>91.560068574442838</v>
       </c>
-      <c r="O24" s="2">
-        <f t="shared" si="0"/>
-        <v>95.59924325732942</v>
-      </c>
-      <c r="P24">
-        <f t="shared" si="1"/>
-        <v>5.2106890676926927</v>
+      <c r="N24" s="4">
+        <v>96.102952898871635</v>
+      </c>
+      <c r="O24" s="1">
+        <f t="shared" si="0"/>
+        <v>93.314727334811849</v>
+      </c>
+      <c r="P24" s="4">
+        <f t="shared" si="1"/>
+        <v>1.993430000368529</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
-        <v>33</v>
+      <c r="A25" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="B25">
         <v>1.5</v>
@@ -1779,30 +1812,30 @@
       <c r="I25">
         <v>2.5</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>86.787284755695254</v>
       </c>
-      <c r="L25">
-        <v>92.662062280382926</v>
-      </c>
-      <c r="M25">
+      <c r="L25" s="4">
         <v>92.362316553574232</v>
       </c>
-      <c r="N25">
+      <c r="M25" s="4">
         <v>84.992746933931159</v>
       </c>
-      <c r="O25" s="2">
-        <f t="shared" si="0"/>
-        <v>90.005708589296091</v>
-      </c>
-      <c r="P25">
-        <f t="shared" si="1"/>
-        <v>3.5468108016267674</v>
+      <c r="N25" s="4">
+        <v>85.517155864170192</v>
+      </c>
+      <c r="O25" s="1">
+        <f t="shared" si="0"/>
+        <v>87.624073117225194</v>
+      </c>
+      <c r="P25" s="4">
+        <f t="shared" si="1"/>
+        <v>3.3572771038553615</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
-        <v>34</v>
+      <c r="A26" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -1828,30 +1861,30 @@
       <c r="I26">
         <v>1</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>89.315285375271145</v>
       </c>
-      <c r="L26">
-        <v>111.41887798376351</v>
-      </c>
-      <c r="M26">
+      <c r="L26" s="4">
         <v>93.985437002637568</v>
       </c>
-      <c r="N26">
+      <c r="M26" s="4">
         <v>93.300804430964007</v>
       </c>
-      <c r="O26" s="2">
-        <f t="shared" si="0"/>
-        <v>99.568373139121675</v>
-      </c>
-      <c r="P26">
-        <f t="shared" si="1"/>
-        <v>8.3842323935749938</v>
+      <c r="N26" s="4">
+        <v>94.636246080810594</v>
+      </c>
+      <c r="O26" s="1">
+        <f t="shared" si="0"/>
+        <v>93.974162504804056</v>
+      </c>
+      <c r="P26" s="4">
+        <f t="shared" si="1"/>
+        <v>0.54525005625082501</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>35</v>
+      <c r="A27" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -1877,30 +1910,30 @@
       <c r="I27">
         <v>1.5</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>86.132089633639836</v>
       </c>
-      <c r="L27">
-        <v>104.87580273839818</v>
-      </c>
-      <c r="M27">
+      <c r="L27" s="4">
         <v>94.147749047543897</v>
       </c>
-      <c r="N27">
+      <c r="M27" s="4">
         <v>92.74693393116182</v>
       </c>
-      <c r="O27" s="2">
-        <f t="shared" si="0"/>
-        <v>97.256828572367965</v>
-      </c>
-      <c r="P27">
-        <f t="shared" si="1"/>
-        <v>5.4176960819489786</v>
+      <c r="N27" s="4">
+        <v>92.404300922891608</v>
+      </c>
+      <c r="O27" s="1">
+        <f t="shared" si="0"/>
+        <v>93.099661300532432</v>
+      </c>
+      <c r="P27" s="4">
+        <f t="shared" si="1"/>
+        <v>0.75419506259576075</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A28" s="1" t="s">
-        <v>36</v>
+      <c r="A28" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="B28">
         <v>0.5</v>
@@ -1926,30 +1959,30 @@
       <c r="I28">
         <v>3.5</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>90.56548060712646</v>
       </c>
-      <c r="L28">
-        <v>103.91615170241127</v>
-      </c>
-      <c r="M28">
+      <c r="L28" s="4">
         <v>97.475145968123712</v>
       </c>
-      <c r="N28">
+      <c r="M28" s="4">
         <v>100.10549914281947</v>
       </c>
-      <c r="O28" s="2">
-        <f t="shared" si="0"/>
-        <v>100.49893227111814</v>
-      </c>
-      <c r="P28">
-        <f t="shared" si="1"/>
-        <v>2.6442051026239075</v>
+      <c r="N28" s="4">
+        <v>87.685331160434345</v>
+      </c>
+      <c r="O28" s="1">
+        <f t="shared" si="0"/>
+        <v>95.088658757125856</v>
+      </c>
+      <c r="P28" s="4">
+        <f t="shared" si="1"/>
+        <v>5.3439457384881468</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
-        <v>37</v>
+      <c r="A29" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -1975,30 +2008,30 @@
       <c r="I29">
         <v>3</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>78.90079227274002</v>
       </c>
-      <c r="L29">
-        <v>86.642433054646801</v>
-      </c>
-      <c r="M29">
+      <c r="L29" s="4">
         <v>78.971572848801813</v>
       </c>
-      <c r="N29">
+      <c r="M29" s="4">
         <v>80.640907292628256</v>
       </c>
-      <c r="O29" s="2">
-        <f t="shared" si="0"/>
-        <v>82.084971065358957</v>
-      </c>
-      <c r="P29">
-        <f t="shared" si="1"/>
-        <v>3.2938846578863861</v>
+      <c r="N29" s="4">
+        <v>77.482153295661888</v>
+      </c>
+      <c r="O29" s="1">
+        <f t="shared" si="0"/>
+        <v>79.031544479030643</v>
+      </c>
+      <c r="P29" s="4">
+        <f t="shared" si="1"/>
+        <v>1.2902529857000862</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
-        <v>38</v>
+      <c r="A30" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="B30">
         <v>0.5</v>
@@ -2024,30 +2057,30 @@
       <c r="I30">
         <v>2</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>90.109249684115497</v>
       </c>
-      <c r="L30">
-        <v>95.977220404701328</v>
-      </c>
-      <c r="M30">
+      <c r="L30" s="4">
         <v>94.634685182262885</v>
       </c>
-      <c r="N30">
+      <c r="M30" s="4">
         <v>88.94896478966109</v>
       </c>
-      <c r="O30" s="2">
-        <f t="shared" si="0"/>
-        <v>93.186956792208434</v>
-      </c>
-      <c r="P30">
-        <f t="shared" si="1"/>
-        <v>3.0464222038443056</v>
+      <c r="N30" s="4">
+        <v>88.833188670221247</v>
+      </c>
+      <c r="O30" s="1">
+        <f t="shared" si="0"/>
+        <v>90.805612880715088</v>
+      </c>
+      <c r="P30" s="4">
+        <f t="shared" si="1"/>
+        <v>2.7079755101451246</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
-        <v>39</v>
+      <c r="A31" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -2073,30 +2106,30 @@
       <c r="I31">
         <v>1</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>88.741803076625303</v>
       </c>
-      <c r="L31">
-        <v>96.936871440688265</v>
-      </c>
-      <c r="M31">
+      <c r="L31" s="4">
         <v>96.663585743592037</v>
       </c>
-      <c r="N31">
+      <c r="M31" s="4">
         <v>94.171172359224585</v>
       </c>
-      <c r="O31" s="2">
-        <f t="shared" si="0"/>
-        <v>95.923876514501629</v>
-      </c>
-      <c r="P31">
-        <f t="shared" si="1"/>
-        <v>1.2443606551166226</v>
+      <c r="N31" s="4">
+        <v>99.227676119958204</v>
+      </c>
+      <c r="O31" s="1">
+        <f t="shared" si="0"/>
+        <v>96.687478074258294</v>
+      </c>
+      <c r="P31" s="4">
+        <f t="shared" si="1"/>
+        <v>2.0643781473972265</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
-        <v>40</v>
+      <c r="A32" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="B32">
         <v>2.5</v>
@@ -2122,30 +2155,30 @@
       <c r="I32">
         <v>6</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>69.702868654977749</v>
       </c>
-      <c r="L32">
-        <v>64.1342542105901</v>
-      </c>
-      <c r="M32">
+      <c r="L32" s="4">
         <v>72.884871164814342</v>
       </c>
-      <c r="N32">
+      <c r="M32" s="4">
         <v>73.203217723855985</v>
       </c>
-      <c r="O32" s="2">
-        <f t="shared" si="0"/>
-        <v>70.074114366420133</v>
-      </c>
-      <c r="P32">
-        <f t="shared" si="1"/>
-        <v>4.2021256633618487</v>
+      <c r="N32" s="4">
+        <v>71.296476715143584</v>
+      </c>
+      <c r="O32" s="1">
+        <f t="shared" si="0"/>
+        <v>72.461521867937961</v>
+      </c>
+      <c r="P32" s="4">
+        <f t="shared" si="1"/>
+        <v>0.83399991564775178</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
-        <v>41</v>
+      <c r="A33" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -2171,30 +2204,30 @@
       <c r="I33">
         <v>2.5</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>94.885461939832865</v>
       </c>
-      <c r="L33">
-        <v>99.641342542105903</v>
-      </c>
-      <c r="M33">
+      <c r="L33" s="4">
         <v>94.391217114903384</v>
       </c>
-      <c r="N33">
+      <c r="M33" s="4">
         <v>87.129104576025313</v>
       </c>
-      <c r="O33" s="2">
-        <f t="shared" si="0"/>
-        <v>93.720554744344881</v>
-      </c>
-      <c r="P33">
-        <f t="shared" si="1"/>
-        <v>5.1300659996676794</v>
+      <c r="N33" s="4">
+        <v>94.636246080810594</v>
+      </c>
+      <c r="O33" s="1">
+        <f t="shared" si="0"/>
+        <v>92.05218925724644</v>
+      </c>
+      <c r="P33" s="4">
+        <f t="shared" si="1"/>
+        <v>3.4825835125080067</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>42</v>
+      <c r="A34" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="B34">
         <v>2</v>
@@ -2220,30 +2253,30 @@
       <c r="I34">
         <v>6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>37.219610311380713</v>
       </c>
-      <c r="L34">
-        <v>47.122258572640256</v>
-      </c>
-      <c r="M34">
+      <c r="L34" s="4">
         <v>34.254604477107229</v>
       </c>
-      <c r="N34">
+      <c r="M34" s="4">
         <v>27.152841883159702</v>
       </c>
-      <c r="O34" s="2">
-        <f t="shared" si="0"/>
-        <v>36.17656831096906</v>
-      </c>
-      <c r="P34">
-        <f t="shared" si="1"/>
-        <v>8.2649807204264327</v>
+      <c r="N34" s="4">
+        <v>33.225869307211312</v>
+      </c>
+      <c r="O34" s="1">
+        <f t="shared" si="0"/>
+        <v>31.54443855582608</v>
+      </c>
+      <c r="P34" s="4">
+        <f t="shared" si="1"/>
+        <v>3.1335991036906217</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
-        <v>43</v>
+      <c r="A35" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -2269,30 +2302,30 @@
       <c r="I35">
         <v>2.5</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>97.313445013232723</v>
       </c>
-      <c r="L35">
-        <v>99.292378529019771</v>
-      </c>
-      <c r="M35">
+      <c r="L35" s="4">
         <v>91.7130683739489</v>
       </c>
-      <c r="N35">
+      <c r="M35" s="4">
         <v>91.639192931557432</v>
       </c>
-      <c r="O35" s="2">
-        <f t="shared" si="0"/>
-        <v>94.214879944842039</v>
-      </c>
-      <c r="P35">
-        <f t="shared" si="1"/>
-        <v>3.5904603511241961</v>
+      <c r="N35" s="4">
+        <v>90.682514658211261</v>
+      </c>
+      <c r="O35" s="1">
+        <f t="shared" si="0"/>
+        <v>91.344925321239202</v>
+      </c>
+      <c r="P35" s="4">
+        <f t="shared" si="1"/>
+        <v>0.46936503925833445</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>44</v>
+      <c r="A36" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="B36">
         <v>1.5</v>
@@ -2318,30 +2351,30 @@
       <c r="I36">
         <v>6</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>24.001403751002378</v>
       </c>
-      <c r="L36">
-        <v>17.722040470132079</v>
-      </c>
-      <c r="M36">
+      <c r="L36" s="4">
         <v>24.434725760274123</v>
       </c>
-      <c r="N36">
+      <c r="M36" s="4">
         <v>26.361598312013715</v>
       </c>
-      <c r="O36" s="2">
-        <f t="shared" si="0"/>
-        <v>22.839454847473306</v>
-      </c>
-      <c r="P36">
-        <f t="shared" si="1"/>
-        <v>3.7030759187217992</v>
+      <c r="N36" s="4">
+        <v>30.802614564327854</v>
+      </c>
+      <c r="O36" s="1">
+        <f t="shared" si="0"/>
+        <v>27.199646212205227</v>
+      </c>
+      <c r="P36" s="4">
+        <f t="shared" si="1"/>
+        <v>2.666363962085168</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
-        <v>45</v>
+      <c r="A37" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -2367,30 +2400,30 @@
       <c r="I37">
         <v>6</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>61.871011501715792</v>
       </c>
-      <c r="L37">
-        <v>68.496304374166982</v>
-      </c>
-      <c r="M37">
+      <c r="L37" s="4">
         <v>78.890416826348627</v>
       </c>
-      <c r="N37">
+      <c r="M37" s="4">
         <v>81.036529078201241</v>
       </c>
-      <c r="O37" s="2">
-        <f t="shared" si="0"/>
-        <v>76.14108342623895</v>
-      </c>
-      <c r="P37">
-        <f t="shared" si="1"/>
-        <v>5.4762173389811544</v>
+      <c r="N37" s="4">
+        <v>67.215205569234584</v>
+      </c>
+      <c r="O37" s="1">
+        <f t="shared" si="0"/>
+        <v>75.714050491261489</v>
+      </c>
+      <c r="P37" s="4">
+        <f t="shared" si="1"/>
+        <v>6.0731223823161891</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
-        <v>46</v>
+      <c r="A38" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="B38">
         <v>1</v>
@@ -2416,30 +2449,30 @@
       <c r="I38">
         <v>6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>80.437406475853564</v>
       </c>
-      <c r="L38">
-        <v>85.246577002302203</v>
-      </c>
-      <c r="M38">
+      <c r="L38" s="4">
         <v>85.707522712414601</v>
       </c>
-      <c r="N38">
+      <c r="M38" s="4">
         <v>81.43215086377424</v>
       </c>
-      <c r="O38" s="2">
-        <f t="shared" si="0"/>
-        <v>84.128750192830339</v>
-      </c>
-      <c r="P38">
-        <f t="shared" si="1"/>
-        <v>1.9160469188787532</v>
+      <c r="N38" s="4">
+        <v>83.859139461144693</v>
+      </c>
+      <c r="O38" s="1">
+        <f t="shared" si="0"/>
+        <v>83.666271012444511</v>
+      </c>
+      <c r="P38" s="4">
+        <f t="shared" si="1"/>
+        <v>1.7507331397473909</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
-        <v>47</v>
+      <c r="A39" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -2465,30 +2498,30 @@
       <c r="I39">
         <v>1</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>80.402018881193641</v>
       </c>
-      <c r="L39">
-        <v>98.507209499575936</v>
-      </c>
-      <c r="M39">
+      <c r="L39" s="4">
         <v>91.7130683739489</v>
       </c>
-      <c r="N39">
+      <c r="M39" s="4">
         <v>90.135830146380059</v>
       </c>
-      <c r="O39" s="2">
-        <f t="shared" si="0"/>
-        <v>93.452036006634955</v>
-      </c>
-      <c r="P39">
-        <f t="shared" si="1"/>
-        <v>3.6320796971272431</v>
+      <c r="N39" s="4">
+        <v>92.723150231165747</v>
+      </c>
+      <c r="O39" s="1">
+        <f t="shared" si="0"/>
+        <v>91.524016250498235</v>
+      </c>
+      <c r="P39" s="4">
+        <f t="shared" si="1"/>
+        <v>1.0646945835370689</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
-        <v>48</v>
+      <c r="A40" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -2514,30 +2547,30 @@
       <c r="I40">
         <v>6</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>72.701010844325083</v>
       </c>
-      <c r="L40">
-        <v>81.407972858354555</v>
-      </c>
-      <c r="M40">
+      <c r="L40" s="4">
         <v>78.24116864672331</v>
       </c>
-      <c r="N40">
+      <c r="M40" s="4">
         <v>85.863114862191736</v>
       </c>
-      <c r="O40" s="2">
-        <f t="shared" si="0"/>
-        <v>81.837418789089867</v>
-      </c>
-      <c r="P40">
-        <f t="shared" si="1"/>
-        <v>3.1264286210138885</v>
+      <c r="N40" s="4">
+        <v>85.198306555896067</v>
+      </c>
+      <c r="O40" s="1">
+        <f t="shared" si="0"/>
+        <v>83.100863354937033</v>
+      </c>
+      <c r="P40" s="4">
+        <f t="shared" si="1"/>
+        <v>3.4470245153185197</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
-        <v>49</v>
+      <c r="A41" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="B41">
         <v>1.5</v>
@@ -2563,28 +2596,28 @@
       <c r="I41">
         <v>6</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>37.313371814019078</v>
       </c>
-      <c r="L41">
-        <v>72.771113534472335</v>
-      </c>
-      <c r="M41">
+      <c r="L41" s="4">
         <v>61.279559954011575</v>
       </c>
-      <c r="N41">
+      <c r="M41" s="4">
         <v>50.573651589080839</v>
       </c>
-      <c r="O41" s="2">
-        <f t="shared" si="0"/>
-        <v>61.54144169252158</v>
-      </c>
-      <c r="P41">
-        <f t="shared" si="1"/>
-        <v>9.0639677013987843</v>
+      <c r="N41" s="4">
+        <v>53.249605866827281</v>
+      </c>
+      <c r="O41" s="1">
+        <f t="shared" si="0"/>
+        <v>55.034272469973224</v>
+      </c>
+      <c r="P41" s="4">
+        <f>_xlfn.STDEV.P(L41:N41)</f>
+        <v>4.5492046662291674</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>